<commit_message>
Sửa: tên sách xuất theo tên đã khai báo, bỏ gộp theo tên
- Tên in ra file: tên khai báo trong danh mục → tên sổ mã chuẩn web → tên thành phần combo → tên tạm (tên sàn – phân loại, có nhãn 'chưa có tên khai báo')
- Chỉ gộp khi cùng barcode (đã quy mã) hoặc SKU trống/chữ cùng tên + phân loại + giá; 2 barcode khác nhau luôn là 2 dòng
- Khớp sổ mã chuẩn và phát hiện tái bản theo tên sàn + phân loại; tên có số khác nhau không bị coi là cùng cuốn
- Khai báo tên: nút sửa trên màn tách đơn, cột Tên sách + lọc 'Chưa có tên khai báo' + lưu hàng loạt ở Danh mục, cột ten_sach trong Excel
- Code.gs: SKU_NHA thêm cột ten_sach, phan_loai (tự thêm tiêu đề cho sheet cũ), action luuTenSach; tự học không ghi đè tên
- Cài đặt: danh sách phân loại vô nghĩa

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016MnyhM5oTNDDoJ5ATt4D6C
</commit_message>
<xml_diff>
--- a/templates/mau-nap-danh-muc.xlsx
+++ b/templates/mau-nap-danh-muc.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A22"/>
   <cols>
     <col min="1" max="1" width="110.83203125" customWidth="1"/>
   </cols>
@@ -432,97 +432,108 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v xml:space="preserve">   - gia_gan_nhat (không bắt buộc): giá gốc gần nhất của cuốn sách – dùng khi tách combo.</v>
+        <v xml:space="preserve">   - ten_sach (Tên sách – không bắt buộc): tên in ra file gửi nhà, ví dụ "Vở BT Thực Hành Mĩ Thuật 3". Cột ten là tên listing trên sàn.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v xml:space="preserve">   - ma_moi (không bắt buộc): sách tái bản đổi mã vạch → ghi mã vạch MỚI vào dòng của mã CŨ.</v>
+        <v xml:space="preserve">     Có cột ten_sach thì ô trống = bỏ tên đã khai báo; không có cột này thì giữ nguyên tên đã khai báo.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v xml:space="preserve">     Nên dùng nút "🔁 Thay mã tái bản" trong app thay vì nạp cột này (app tự đổi luôn thành phần combo).</v>
+        <v xml:space="preserve">   - gia_gan_nhat (không bắt buộc): giá gốc gần nhất của cuốn sách – dùng khi tách combo.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2. Sheet COMBO: mỗi dòng 1 combo. combo_id tự đặt (ví dụ C001), không trùng nhau.</v>
+        <v xml:space="preserve">   - ma_moi (không bắt buộc): sách tái bản đổi mã vạch → ghi mã vạch MỚI vào dòng của mã CŨ.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v xml:space="preserve">   - Cột khoa: SKU của combo trên các sàn, cách nhau bằng " ;; " (ví dụ: 55252 ;; 8935092825724|COMBO.HA).</v>
+        <v xml:space="preserve">     Nên dùng nút "🔁 Thay mã tái bản" trong app thay vì nạp cột này (app tự đổi luôn thành phần combo).</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v xml:space="preserve">   - Combo có SKU là MÃ VẠCH (mã của 1 cuốn lẻ): ghi &lt;mã vạch&gt;|&lt;phân loại&gt; (ví dụ 8935092825724|COMBO.HA).</v>
+        <v>2. Sheet COMBO: mỗi dòng 1 combo. combo_id tự đặt (ví dụ C001), không trùng nhau.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v xml:space="preserve">   - Combo không có SKU: ghi ten:&lt;tên sản phẩm&gt;|&lt;phân loại&gt; (chữ thường).</v>
+        <v xml:space="preserve">   - Cột khoa: SKU của combo trên các sàn, cách nhau bằng " ;; " (ví dụ: 55252 ;; 8935092825724|COMBO.HA).</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v xml:space="preserve">   - Cột cach_xuat: tach = tách thành từng cuốn (mặc định) ; nguyen = xuất nguyên combo thành 1 dòng.</v>
+        <v xml:space="preserve">   - Combo có SKU là MÃ VẠCH (mã của 1 cuốn lẻ): ghi &lt;mã vạch&gt;|&lt;phân loại&gt; (ví dụ 8935092825724|COMBO.HA).</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v xml:space="preserve">   - Combo "nguyen": cần cột nha (HA / KV / ML), không cần thành phần. ma_he_thong = mã combo trên website lên đơn</v>
+        <v xml:space="preserve">   - Combo không có SKU: ghi ten:&lt;tên sản phẩm&gt;|&lt;phân loại&gt; (chữ thường).</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v xml:space="preserve">     (để trống = dùng SKU của sàn). ten_xuat = tên in ra file (để trống = tên combo đã làm gọn).</v>
+        <v xml:space="preserve">   - Cột cach_xuat: tach = tách thành từng cuốn (mặc định) ; nguyen = xuất nguyên combo thành 1 dòng.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>3. Sheet COMBO_THANH_PHAN: mỗi dòng 1 cuốn trong combo, combo_id phải khớp sheet COMBO.</v>
+        <v xml:space="preserve">   - Combo "nguyen": cần cột nha (HA / KV / ML), không cần thành phần. ma_he_thong = mã combo trên website lên đơn</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v xml:space="preserve">   - nha = HA / KV / ML / KHAC (KHAC = sách nhà khác, sẽ không nhập).</v>
+        <v xml:space="preserve">     (để trống = dùng SKU của sàn). ten_xuat = tên in ra file (để trống = tên combo đã làm gọn).</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v xml:space="preserve">   - so_luong = số cuốn đó trong 1 combo (thường là 1).</v>
+        <v>3. Sheet COMBO_THANH_PHAN: mỗi dòng 1 cuốn trong combo, combo_id phải khớp sheet COMBO.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>4. Dòng mẫu bên dưới chỉ để tham khảo – xóa hoặc sửa trước khi nạp.</v>
+        <v xml:space="preserve">   - nha = HA / KV / ML / KHAC (KHAC = sách nhà khác, sẽ không nhập).</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
+        <v xml:space="preserve">   - so_luong = số cuốn đó trong 1 combo (thường là 1).</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>4. Dòng mẫu bên dưới chỉ để tham khảo – xóa hoặc sửa trước khi nạp.</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
         <v>5. Nạp trùng SKU / combo_id đã có thì sẽ GHI ĐÈ dòng cũ.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A20"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A22"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H4"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="60.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="40.83203125" customWidth="1"/>
+    <col min="4" max="4" width="60.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -533,18 +544,21 @@
         <v>sku</v>
       </c>
       <c r="C1" t="str">
+        <v>ten_sach</v>
+      </c>
+      <c r="D1" t="str">
         <v>ten</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>phan_loai</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>nha</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>gia_gan_nhat</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>ma_moi</v>
       </c>
     </row>
@@ -556,18 +570,21 @@
         <v>8935092845425</v>
       </c>
       <c r="C2" t="str">
+        <v>Hướng Dẫn Giải VIOLYMPIC Toán 1</v>
+      </c>
+      <c r="D2" t="str">
         <v>Sách - Hướng Dẫn Giải VIOLYMPIC Toán 1</v>
       </c>
-      <c r="D2" t="str">
-        <v/>
-      </c>
       <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
         <v>HA</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>48000</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v/>
       </c>
     </row>
@@ -579,18 +596,21 @@
         <v>8935092543000</v>
       </c>
       <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
         <v>Sách - Bồi Dưỡng Học Sinh Giỏi Lịch Sử 9</v>
       </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
       <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
         <v>KV</v>
       </c>
-      <c r="F3" t="str">
-        <v/>
-      </c>
       <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
         <v/>
       </c>
     </row>
@@ -602,24 +622,27 @@
         <v/>
       </c>
       <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
         <v>Sách - Ví Dụ Sách Không Có Mã Vạch - Newshop</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>Mặc định</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>KHONG_NHAP</v>
       </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
       <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Sửa / bổ sung barcode cho từng dòng (nút 🏷️)
- Nút 🏷️ cạnh ✏️ ở bảng nhà (cả cuốn tách từ combo), Chưa rõ nhà, Đã bỏ qua
- Hộp sửa barcode: tìm theo tên (sổ mã chuẩn web + danh mục, không dấu), cảnh báo sai số kiểm tra EAN-13, hỏi nhà + tên khi barcode mới
- SKU trống / SKU chữ → ánh xạ khóa dòng → barcode; barcode sai → mã phụ; thành phần combo chưa có SKU → điền barcode
- Code.gs: action ganBarcode / boGanBarcode (ảnh chụp trước/sau, hoàn tác được), hỏi trước khi ghi đè ánh xạ gán tay
- Danh mục: tab "Barcode gán tay" (sửa / bỏ, tìm không dấu); Excel có sheet BARCODE_GAN_TAY
- Dòng vừa gán / sửa vào "Listing cần sửa barcode"

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016MnyhM5oTNDDoJ5ATt4D6C
</commit_message>
<xml_diff>
--- a/templates/mau-nap-danh-muc.xlsx
+++ b/templates/mau-nap-danh-muc.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A25"/>
   <cols>
     <col min="1" max="1" width="110.83203125" customWidth="1"/>
   </cols>
@@ -515,9 +515,24 @@
         <v>5. Nạp trùng SKU / combo_id đã có thì sẽ GHI ĐÈ dòng cũ.</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>6. Sheet BARCODE_GAN_TAY (không bắt buộc): dòng trên sàn có SKU trống / SKU chữ / barcode sai → barcode đúng.</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v xml:space="preserve">   - Có SKU (chữ hoặc barcode sai): điền sku_tren_san. SKU trống: điền ten_tren_san + phan_loai ĐÚNG như trên sàn.</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v xml:space="preserve">   - barcode_dung: mã vạch đúng. Nạp trùng khóa thì ghi đè barcode cũ.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A25"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>